<commit_message>
feat: Include self id when movement is done
- Added id when user do a movement
- Added new dependency to manage the excel template and replace basic data
- Fixed bugs on report endpoints
</commit_message>
<xml_diff>
--- a/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
+++ b/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebav\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebav\OneDrive\Documentos\Github\DISERCO-Inventory\Backend\internal\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A3023B-2E0A-46F1-9727-157853C4BA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4905952-291D-4C28-933F-463300C612CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="577" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="577" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen General" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="24">
   <si>
     <t>REPORTE GENERAL DE ABASTECIMIENTO</t>
   </si>
@@ -203,35 +203,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,22 +539,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="16"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -564,7 +560,6 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -580,7 +575,6 @@
       <c r="E4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -592,7 +586,6 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -604,7 +597,6 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
@@ -612,35 +604,34 @@
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="F7" s="11"/>
     </row>
     <row r="8" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="17"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="12"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -658,97 +649,47 @@
       <c r="E10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="13"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="13"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="13"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="10"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="13"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="10"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="13"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -768,24 +709,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -832,36 +773,36 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="11" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implemented excel reports
- Refactored code to accept decimals
- Excel report can be generate with general summary and summary for each section.
</commit_message>
<xml_diff>
--- a/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
+++ b/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebav\OneDrive\Documentos\Github\DISERCO-Inventory\Backend\internal\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4905952-291D-4C28-933F-463300C612CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62891BEA-EB3A-4EC7-A527-2E6E46660025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="577" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>REPORTE GENERAL DE ABASTECIMIENTO</t>
   </si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>Salidas</t>
-  </si>
-  <si>
-    <t>{{dato}}</t>
   </si>
   <si>
     <t>DETALLE DE ABASTECIMIENTO POR SECCIÓN</t>
@@ -99,7 +96,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +142,11 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -229,7 +231,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -570,10 +572,10 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -634,61 +636,51 @@
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
       <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
       <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
       <c r="F12" s="10"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="10"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
       <c r="F14" s="10"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
       <c r="F15" s="10"/>
     </row>
   </sheetData>
@@ -710,7 +702,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -742,7 +734,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -774,7 +766,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -785,10 +777,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>11</v>
@@ -797,359 +789,149 @@
         <v>12</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>23</v>
-      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Refactor: Export report template and function changed
- Report now contains all items in a sheet instead of different sheet with only the movements items
- Fixed InventoryItemService to create movements (entry/exit) without the ID "1" (default id)
- Removed unused entities
</commit_message>
<xml_diff>
--- a/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
+++ b/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
@@ -8,20 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebav\OneDrive\Documentos\Github\DISERCO-Inventory\Backend\internal\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62891BEA-EB3A-4EC7-A527-2E6E46660025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAAEFF8C-E195-4079-870A-6CE702E7088C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="577" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="577" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen General" sheetId="1" r:id="rId1"/>
-    <sheet name="Detalle Sección" sheetId="2" r:id="rId2"/>
+    <sheet name="Inventario Detallado" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventario Detallado'!$A$8:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen General'!$A$9:$E$9</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>REPORTE GENERAL DE ABASTECIMIENTO</t>
   </si>
@@ -62,12 +66,6 @@
     <t>Salidas</t>
   </si>
   <si>
-    <t>DETALLE DE ABASTECIMIENTO POR SECCIÓN</t>
-  </si>
-  <si>
-    <t>{{seccion_nombre}}</t>
-  </si>
-  <si>
     <t>Detalle de Materiales y Herramientas</t>
   </si>
   <si>
@@ -83,13 +81,19 @@
     <t>{{n_reporte}}</t>
   </si>
   <si>
-    <t>Observacion</t>
-  </si>
-  <si>
     <t>Stock disponible</t>
   </si>
   <si>
     <t>Responsable/s</t>
+  </si>
+  <si>
+    <t>Observación</t>
+  </si>
+  <si>
+    <t>DETALLE DE INVENTARIO DE TODAS LAS SECCIÓN</t>
+  </si>
+  <si>
+    <t>Inventario total hasta el dia:</t>
   </si>
 </sst>
 </file>
@@ -205,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -225,13 +229,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,20 +551,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -572,10 +582,10 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -608,13 +618,13 @@
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
       <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -636,11 +646,11 @@
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
       <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -684,6 +694,7 @@
       <c r="F15" s="10"/>
     </row>
   </sheetData>
+  <autoFilter ref="A9:E9" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A1:E2"/>
@@ -694,33 +705,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="20" customWidth="1"/>
+    <col min="1" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-    </row>
-    <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -728,34 +741,33 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="D5" s="16"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -763,10 +775,11 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -774,31 +787,35 @@
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="8"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -806,8 +823,9 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -816,7 +834,7 @@
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -825,7 +843,7 @@
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -834,7 +852,7 @@
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -843,7 +861,7 @@
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -852,7 +870,7 @@
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -861,7 +879,7 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -934,8 +952,11 @@
       <c r="G23" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G2"/>
+  <autoFilter ref="A8:H8" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: Auth fields separated
- Changes to reports: rows with deleted or removed items now appear in red.
- Fixed problem when an item is recently added and not appear in maintenance view.
</commit_message>
<xml_diff>
--- a/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
+++ b/Backend/internal/utils/Plantilla_Reporte_Abastecimiento.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebav\OneDrive\Documentos\Github\DISERCO-Inventory\Backend\internal\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAAEFF8C-E195-4079-870A-6CE702E7088C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1852F520-734C-4E59-AE75-0CDD44CA457C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="577" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>REPORTE GENERAL DE ABASTECIMIENTO</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>Inventario total hasta el dia:</t>
+  </si>
+  <si>
+    <t>Elemento eliminado/dado de baja</t>
   </si>
 </sst>
 </file>
@@ -156,7 +159,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -181,8 +184,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -205,11 +214,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -225,9 +247,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -241,6 +260,17 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -551,20 +581,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -618,14 +648,14 @@
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="12"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="11"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
@@ -646,11 +676,11 @@
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -705,35 +735,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
+    <col min="11" max="11" width="26.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -743,7 +774,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="2"/>
@@ -753,21 +784,21 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="16"/>
+      <c r="D5" s="15"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -777,7 +808,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
@@ -788,34 +819,39 @@
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="J7" s="17"/>
+      <c r="K7" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" s="18"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -825,16 +861,17 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -843,7 +880,7 @@
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -852,7 +889,7 @@
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -861,7 +898,7 @@
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -870,7 +907,7 @@
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -879,7 +916,7 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -953,10 +990,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A8:H8" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="K7:L7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>